<commit_message>
[ADDS] pyro pins test
</commit_message>
<xml_diff>
--- a/flight-computer-pin-assignment-version-1.xlsx
+++ b/flight-computer-pin-assignment-version-1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\5th-year\project\N4-Flight-Software\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25662C86-529C-44F5-8C22-486A599FC5D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E7695C4-34E6-46AB-8AE2-AAEB699BDF6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10305" yWindow="495" windowWidth="11925" windowHeight="12405" xr2:uid="{C1B70286-B989-4919-B8D9-1F40D54E6E76}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="12000" windowHeight="13050" xr2:uid="{C1B70286-B989-4919-B8D9-1F40D54E6E76}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -381,7 +381,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -416,7 +416,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1230,7 +1229,7 @@
       <c r="C38" t="s">
         <v>78</v>
       </c>
-      <c r="D38" s="14" t="s">
+      <c r="D38" s="6" t="s">
         <v>74</v>
       </c>
       <c r="E38" s="6" t="s">

</xml_diff>